<commit_message>
Include section in figure file names to avoid Section A/B collisions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NrCi6LsQYkupC3LrqmAUV3
</commit_message>
<xml_diff>
--- a/output/JEE_Questions.xlsx
+++ b/output/JEE_Questions.xlsx
@@ -973,7 +973,7 @@
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-02-24_M/PHY_Q03_1.png</t>
+          <t>figures/JEEM_2021-02-24_M/PHY_A03_1.png</t>
         </is>
       </c>
       <c r="W4" s="2" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="V6" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-02-24_M/PHY_Q05_1.png</t>
+          <t>figures/JEEM_2021-02-24_M/PHY_A05_1.png</t>
         </is>
       </c>
       <c r="W6" s="2" t="inlineStr">
@@ -1596,7 +1596,7 @@
       </c>
       <c r="V9" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-02-24_M/PHY_Q08_1.png</t>
+          <t>figures/JEEM_2021-02-24_M/PHY_A08_1.png</t>
         </is>
       </c>
       <c r="W9" s="2" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="V13" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-02-24_M/PHY_Q12_1.png</t>
+          <t>figures/JEEM_2021-02-24_M/PHY_A12_1.png</t>
         </is>
       </c>
       <c r="W13" s="2" t="inlineStr">
@@ -2846,7 +2846,7 @@
       </c>
       <c r="V19" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-02-24_M/PHY_Q18_1.png</t>
+          <t>figures/JEEM_2021-02-24_M/PHY_A18_1.png</t>
         </is>
       </c>
       <c r="W19" s="2" t="inlineStr">
@@ -2973,7 +2973,7 @@
       </c>
       <c r="V20" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-02-24_M/PHY_Q19_1.png</t>
+          <t>figures/JEEM_2021-02-24_M/PHY_A19_1.png</t>
         </is>
       </c>
       <c r="W20" s="2" t="inlineStr">
@@ -4170,7 +4170,7 @@
       </c>
       <c r="V31" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-02-24_M/PHY_Q10_1.png</t>
+          <t>figures/JEEM_2021-02-24_M/PHY_B10_1.png</t>
         </is>
       </c>
       <c r="W31" s="2" t="inlineStr">
@@ -4671,7 +4671,7 @@
       </c>
       <c r="V35" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-02-24_M/CHE_Q04_1.png</t>
+          <t>figures/JEEM_2021-02-24_M/CHE_A04_1.png</t>
         </is>
       </c>
       <c r="W35" s="2" t="inlineStr">
@@ -4798,7 +4798,7 @@
       </c>
       <c r="V36" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-02-24_M/CHE_Q05_1.png</t>
+          <t>figures/JEEM_2021-02-24_M/CHE_A05_1.png</t>
         </is>
       </c>
       <c r="W36" s="2" t="inlineStr">
@@ -5053,7 +5053,7 @@
       </c>
       <c r="V38" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-02-24_M/CHE_Q07_1.png</t>
+          <t>figures/JEEM_2021-02-24_M/CHE_A07_1.png</t>
         </is>
       </c>
       <c r="W38" s="2" t="inlineStr">
@@ -5429,7 +5429,7 @@
       </c>
       <c r="V41" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-02-24_M/CHE_Q10_1.png</t>
+          <t>figures/JEEM_2021-02-24_M/CHE_A10_1.png</t>
         </is>
       </c>
       <c r="W41" s="2" t="inlineStr">
@@ -5808,7 +5808,7 @@
       </c>
       <c r="V44" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-02-24_M/CHE_Q13_1.png</t>
+          <t>figures/JEEM_2021-02-24_M/CHE_A13_1.png</t>
         </is>
       </c>
       <c r="W44" s="2" t="inlineStr">
@@ -6059,7 +6059,7 @@
       </c>
       <c r="V46" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-02-24_M/CHE_Q15_1.png</t>
+          <t>figures/JEEM_2021-02-24_M/CHE_A15_1.png</t>
         </is>
       </c>
       <c r="W46" s="2" t="inlineStr">
@@ -6186,7 +6186,7 @@
       </c>
       <c r="V47" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-02-24_M/CHE_Q16_1.png</t>
+          <t>figures/JEEM_2021-02-24_M/CHE_A16_1.png</t>
         </is>
       </c>
       <c r="W47" s="2" t="inlineStr">
@@ -12173,7 +12173,7 @@
       </c>
       <c r="V98" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-07-20_M/PHY_Q07_1.png</t>
+          <t>figures/JEEM_2021-07-20_M/PHY_A07_1.png</t>
         </is>
       </c>
       <c r="W98" s="2" t="inlineStr">
@@ -12423,7 +12423,7 @@
       </c>
       <c r="V100" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-07-20_M/PHY_Q09_1.png</t>
+          <t>figures/JEEM_2021-07-20_M/PHY_A09_1.png</t>
         </is>
       </c>
       <c r="W100" s="2" t="inlineStr">
@@ -12550,7 +12550,7 @@
       </c>
       <c r="V101" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-07-20_M/PHY_Q10_1.png</t>
+          <t>figures/JEEM_2021-07-20_M/PHY_A10_1.png</t>
         </is>
       </c>
       <c r="W101" s="2" t="inlineStr">
@@ -12678,7 +12678,7 @@
       </c>
       <c r="V102" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-07-20_M/PHY_Q11_1.png</t>
+          <t>figures/JEEM_2021-07-20_M/PHY_A11_1.png</t>
         </is>
       </c>
       <c r="W102" s="2" t="inlineStr">
@@ -13667,7 +13667,7 @@
       </c>
       <c r="V110" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-07-20_M/PHY_Q19_1.png</t>
+          <t>figures/JEEM_2021-07-20_M/PHY_A19_1.png</t>
         </is>
       </c>
       <c r="W110" s="2" t="inlineStr">
@@ -13794,7 +13794,7 @@
       </c>
       <c r="V111" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-07-20_M/PHY_Q20_1.png</t>
+          <t>figures/JEEM_2021-07-20_M/PHY_A20_1.png</t>
         </is>
       </c>
       <c r="W111" s="2" t="inlineStr">
@@ -14013,7 +14013,7 @@
       </c>
       <c r="V113" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-07-20_M/PHY_Q02_1.png</t>
+          <t>figures/JEEM_2021-07-20_M/PHY_B02_1.png</t>
         </is>
       </c>
       <c r="W113" s="2" t="inlineStr">
@@ -14124,7 +14124,7 @@
       </c>
       <c r="V114" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-07-20_M/PHY_Q03_1.png</t>
+          <t>figures/JEEM_2021-07-20_M/PHY_B03_1.png</t>
         </is>
       </c>
       <c r="W114" s="2" t="inlineStr">
@@ -14342,7 +14342,7 @@
       </c>
       <c r="V116" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-07-20_M/PHY_Q05_1.png</t>
+          <t>figures/JEEM_2021-07-20_M/PHY_B05_1.png</t>
         </is>
       </c>
       <c r="W116" s="2" t="inlineStr">
@@ -15377,7 +15377,7 @@
       </c>
       <c r="V125" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-07-20_M/CHE_Q04_1.png</t>
+          <t>figures/JEEM_2021-07-20_M/CHE_A04_1.png</t>
         </is>
       </c>
       <c r="W125" s="2" t="inlineStr">
@@ -16742,7 +16742,7 @@
       </c>
       <c r="V136" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-07-20_M/CHE_Q15_1.png</t>
+          <t>figures/JEEM_2021-07-20_M/CHE_A15_1.png</t>
         </is>
       </c>
       <c r="W136" s="2" t="inlineStr">
@@ -16993,7 +16993,7 @@
       </c>
       <c r="V138" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-07-20_M/CHE_Q17_1.png</t>
+          <t>figures/JEEM_2021-07-20_M/CHE_A17_1.png</t>
         </is>
       </c>
       <c r="W138" s="2" t="inlineStr">
@@ -17246,7 +17246,7 @@
       </c>
       <c r="V140" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-07-20_M/CHE_Q19_1.png</t>
+          <t>figures/JEEM_2021-07-20_M/CHE_A19_1.png</t>
         </is>
       </c>
       <c r="W140" s="2" t="inlineStr">
@@ -22229,7 +22229,7 @@
       </c>
       <c r="V183" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-08-26_M/PHY_Q02_1.png</t>
+          <t>figures/JEEM_2021-08-26_M/PHY_A02_1.png</t>
         </is>
       </c>
       <c r="W183" s="2" t="inlineStr">
@@ -23100,7 +23100,7 @@
       </c>
       <c r="V190" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-08-26_M/PHY_Q09_1.png</t>
+          <t>figures/JEEM_2021-08-26_M/PHY_A09_1.png</t>
         </is>
       </c>
       <c r="W190" s="2" t="inlineStr">
@@ -23473,7 +23473,7 @@
       </c>
       <c r="V193" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-08-26_M/PHY_Q12_1.png</t>
+          <t>figures/JEEM_2021-08-26_M/PHY_A12_1.png</t>
         </is>
       </c>
       <c r="W193" s="2" t="inlineStr">
@@ -23600,7 +23600,7 @@
       </c>
       <c r="V194" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-08-26_M/PHY_Q13_1.png; figures/JEEM_2021-08-26_M/PHY_Q13_2.png</t>
+          <t>figures/JEEM_2021-08-26_M/PHY_A13_1.png; figures/JEEM_2021-08-26_M/PHY_A13_2.png</t>
         </is>
       </c>
       <c r="W194" s="2" t="inlineStr">
@@ -25223,7 +25223,7 @@
       </c>
       <c r="V208" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-08-26_M/PHY_Q07_1.png</t>
+          <t>figures/JEEM_2021-08-26_M/PHY_B07_1.png</t>
         </is>
       </c>
       <c r="W208" s="2" t="inlineStr">
@@ -25551,7 +25551,7 @@
       </c>
       <c r="V211" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-08-26_M/PHY_Q10_1.png</t>
+          <t>figures/JEEM_2021-08-26_M/PHY_B10_1.png</t>
         </is>
       </c>
       <c r="W211" s="2" t="inlineStr">
@@ -26048,7 +26048,7 @@
       </c>
       <c r="V215" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-08-26_M/CHE_Q04_1.png</t>
+          <t>figures/JEEM_2021-08-26_M/CHE_A04_1.png</t>
         </is>
       </c>
       <c r="W215" s="2" t="inlineStr">
@@ -26176,7 +26176,7 @@
       </c>
       <c r="V216" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-08-26_M/CHE_Q05_1.png</t>
+          <t>figures/JEEM_2021-08-26_M/CHE_A05_1.png</t>
         </is>
       </c>
       <c r="W216" s="2" t="inlineStr">
@@ -26304,7 +26304,7 @@
       </c>
       <c r="V217" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-08-26_M/CHE_Q06_1.png</t>
+          <t>figures/JEEM_2021-08-26_M/CHE_A06_1.png</t>
         </is>
       </c>
       <c r="W217" s="2" t="inlineStr">
@@ -26681,7 +26681,7 @@
       </c>
       <c r="V220" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-08-26_M/CHE_Q09_1.png</t>
+          <t>figures/JEEM_2021-08-26_M/CHE_A09_1.png</t>
         </is>
       </c>
       <c r="W220" s="2" t="inlineStr">
@@ -27058,7 +27058,7 @@
       </c>
       <c r="V223" s="3" t="inlineStr">
         <is>
-          <t>figures/JEEM_2021-08-26_M/CHE_Q12_1.png</t>
+          <t>figures/JEEM_2021-08-26_M/CHE_A12_1.png</t>
         </is>
       </c>
       <c r="W223" s="2" t="inlineStr">

</xml_diff>